<commit_message>
Improve readability of demo database spreadsheet
</commit_message>
<xml_diff>
--- a/demo-database.xlsx
+++ b/demo-database.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Демо-профили" sheetId="1" r:id="R7f61a3b64624451f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Демо-профили" sheetId="1" r:id="R07d92f46f5514611"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -375,7 +375,7 @@
         <x:v>Ограничения</x:v>
       </x:c>
       <x:c r="I2" s="10" t="str">
-        <x:v>Фото / файл</x:v>
+        <x:v>Фото (имя файла)</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="42" customHeight="1">
@@ -507,7 +507,7 @@
     </x:row>
     <x:row r="8" ht="58" customHeight="1">
       <x:c r="A8" s="16" t="str">
-        <x:v>Схема: accounts(id, name, company, work_scope, site, access_until, status, restrictions, photo_url). ID и профиль — демонстрационные. Фото являются визуальными примерами персонажей, не подтверждают личность и не подходят для реального допуска.</x:v>
+        <x:v>Схема: accounts(id, name, company, work_scope, site, access_until, status, restrictions, photo_url). ID и профиль — демонстрационные. Фото — иллюстрации персонажей; не подтверждают личность. Файлы с одинаковыми именами находятся в avatars/ приложения и docs/checker/.</x:v>
       </x:c>
       <x:c r="B8" s="16"/>
       <x:c r="C8" s="16"/>

</xml_diff>

<commit_message>
Add readable photo filenames to demo spreadsheet
</commit_message>
<xml_diff>
--- a/demo-database.xlsx
+++ b/demo-database.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Демо-профили" sheetId="1" r:id="R07d92f46f5514611"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Демо-профили" sheetId="1" r:id="Rf9acbe2b64984426"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -333,7 +333,7 @@
     <x:col min="6" max="6" width="8.380000114440918" hidden="0" customWidth="1"/>
     <x:col min="7" max="7" width="12.380000114440918" hidden="0" customWidth="1"/>
     <x:col min="8" max="8" width="28.6299991607666" hidden="0" customWidth="1"/>
-    <x:col min="9" max="9" width="53.25" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="17.6299991607666" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="30" customHeight="1">
@@ -404,7 +404,7 @@
         <x:v>Без дополнительных ограничений</x:v>
       </x:c>
       <x:c r="I3" s="11" t="str">
-        <x:v>app/src/main/assets/avatars/TP-0001.png; docs/checker/avatars/TP-0001.png</x:v>
+        <x:v>TP-0001.png — APK + QR</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="42" customHeight="1">
@@ -433,7 +433,7 @@
         <x:v>Только АПС; требуется ручная проверка</x:v>
       </x:c>
       <x:c r="I4" s="11" t="str">
-        <x:v>app/src/main/assets/avatars/TP-0002.png; docs/checker/avatars/TP-0002.png</x:v>
+        <x:v>TP-0002.png — APK + QR</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="42" customHeight="1">
@@ -462,7 +462,7 @@
         <x:v>Продлить допуск перед работами</x:v>
       </x:c>
       <x:c r="I5" s="11" t="str">
-        <x:v>app/src/main/assets/avatars/TP-0003.png; docs/checker/avatars/TP-0003.png</x:v>
+        <x:v>TP-0003.png — APK + QR</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="42" customHeight="1">
@@ -491,7 +491,7 @@
         <x:v>Доступ отозван ответственным</x:v>
       </x:c>
       <x:c r="I6" s="11" t="str">
-        <x:v>app/src/main/assets/avatars/TP-0004.png; docs/checker/avatars/TP-0004.png</x:v>
+        <x:v>TP-0004.png — APK + QR</x:v>
       </x:c>
     </x:row>
     <x:row r="7">

</xml_diff>

<commit_message>
Replace damaged demo portraits with optimized JPG assets
</commit_message>
<xml_diff>
--- a/demo-database.xlsx
+++ b/demo-database.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Демо-профили" sheetId="1" r:id="Rf9acbe2b64984426"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Демо-профили" sheetId="1" r:id="R5ba725371628486a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -333,7 +333,7 @@
     <x:col min="6" max="6" width="8.380000114440918" hidden="0" customWidth="1"/>
     <x:col min="7" max="7" width="12.380000114440918" hidden="0" customWidth="1"/>
     <x:col min="8" max="8" width="28.6299991607666" hidden="0" customWidth="1"/>
-    <x:col min="9" max="9" width="17.6299991607666" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="17.1299991607666" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="30" customHeight="1">
@@ -404,7 +404,7 @@
         <x:v>Без дополнительных ограничений</x:v>
       </x:c>
       <x:c r="I3" s="11" t="str">
-        <x:v>TP-0001.png — APK + QR</x:v>
+        <x:v>TP-0001.jpg — APK + QR</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="42" customHeight="1">
@@ -433,7 +433,7 @@
         <x:v>Только АПС; требуется ручная проверка</x:v>
       </x:c>
       <x:c r="I4" s="11" t="str">
-        <x:v>TP-0002.png — APK + QR</x:v>
+        <x:v>TP-0002.jpg — APK + QR</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="42" customHeight="1">
@@ -462,7 +462,7 @@
         <x:v>Продлить допуск перед работами</x:v>
       </x:c>
       <x:c r="I5" s="11" t="str">
-        <x:v>TP-0003.png — APK + QR</x:v>
+        <x:v>TP-0003.jpg — APK + QR</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="42" customHeight="1">
@@ -491,7 +491,7 @@
         <x:v>Доступ отозван ответственным</x:v>
       </x:c>
       <x:c r="I6" s="11" t="str">
-        <x:v>TP-0004.png — APK + QR</x:v>
+        <x:v>TP-0004.jpg — APK + QR</x:v>
       </x:c>
     </x:row>
     <x:row r="7">

</xml_diff>